<commit_message>
begin providing support for "Reports" reference type.
</commit_message>
<xml_diff>
--- a/inst/extdata/DSbulkUploadR_input.xlsx
+++ b/inst/extdata/DSbulkUploadR_input.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rlbaker\Rdev_local\DSbulkUploadR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B5CCE8-5636-4B82-91A9-0450FC349CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2318D46F-8307-4193-A3D2-96A9F47D0BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28755" yWindow="1935" windowWidth="26325" windowHeight="8145" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
+    <workbookView xWindow="37470" yWindow="3210" windowWidth="23010" windowHeight="12210" activeTab="1" xr2:uid="{8A6EE447-C162-4970-95C2-F79FBBAD4C55}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="5" r:id="rId1"/>
-    <sheet name="GenericDataset" sheetId="4" r:id="rId2"/>
-    <sheet name="FieldNotes" sheetId="6" r:id="rId3"/>
-    <sheet name="GenericDocument" sheetId="2" r:id="rId4"/>
-    <sheet name="AudioRecording" sheetId="1" r:id="rId5"/>
-    <sheet name="Script" sheetId="7" r:id="rId6"/>
-    <sheet name="WebSite" sheetId="3" r:id="rId7"/>
+    <sheet name="Reports" sheetId="8" r:id="rId2"/>
+    <sheet name="GenericDataset" sheetId="4" r:id="rId3"/>
+    <sheet name="FieldNotes" sheetId="6" r:id="rId4"/>
+    <sheet name="GenericDocument" sheetId="2" r:id="rId5"/>
+    <sheet name="AudioRecording" sheetId="1" r:id="rId6"/>
+    <sheet name="Script" sheetId="7" r:id="rId7"/>
+    <sheet name="WebSite" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="89">
   <si>
     <t>reference_type</t>
   </si>
@@ -300,6 +301,15 @@
   </si>
   <si>
     <t>robert_baker@nps.gov</t>
+  </si>
+  <si>
+    <t>date_published</t>
+  </si>
+  <si>
+    <t>publisher</t>
+  </si>
+  <si>
+    <t>National Park Service</t>
   </si>
 </sst>
 </file>
@@ -806,6 +816,133 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9481F28-1651-4F2B-B124-AF1022AC39C7}">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="1">
+        <v>44331</v>
+      </c>
+      <c r="F2" t="s">
+        <v>88</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q2">
+        <v>2315517</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C2" xr:uid="{E08A2139-E969-40A7-8EEC-53BB78CF21E3}">
+      <formula1>"Yes, No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1" xr:uid="{55D934E0-4744-4F13-8FC1-B58643BAA9FE}">
+      <formula1>"GenericDocument"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{56886875-4262-4C01-B9B5-18A23F6DE832}">
+      <formula1>"PublishedReport"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B81407D-D8D8-4DE4-AB2A-A11A6520C285}">
   <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -952,7 +1089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02740E3C-2CB5-4540-B9FC-9B8FBF6E48A3}">
   <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1209,7 +1346,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32C372F4-B2F9-43E8-90EB-ACDD3F5DA605}">
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1415,7 +1552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AA704E2-EB95-4E4A-95B2-36E8F6DDD1DD}">
   <dimension ref="A1:T3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1637,7 +1774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D704E2B-E668-4D16-AAE0-B58A99B5B51C}">
   <dimension ref="A1:T3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1847,7 +1984,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0591C5C5-FA56-4654-9944-818D77B92433}">
   <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>